<commit_message>
chat initiation and send message feature done
</commit_message>
<xml_diff>
--- a/schema/schema_design.xlsx
+++ b/schema/schema_design.xlsx
@@ -119,7 +119,7 @@
     <t>group_users</t>
   </si>
   <si>
-    <t>conversation</t>
+    <t>conversations</t>
   </si>
   <si>
     <t>group_id</t>
@@ -1999,17 +1999,17 @@
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="F21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>

</xml_diff>

<commit_message>
some support changes done
</commit_message>
<xml_diff>
--- a/schema/schema_design.xlsx
+++ b/schema/schema_design.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="41">
   <si>
     <t>users</t>
   </si>
@@ -107,10 +107,16 @@
     <t>updated_on</t>
   </si>
   <si>
+    <t>display_name</t>
+  </si>
+  <si>
     <t>profile_image_url</t>
   </si>
   <si>
     <t>activity_type</t>
+  </si>
+  <si>
+    <t>chat_read</t>
   </si>
   <si>
     <t>chat_groups</t>
@@ -1562,17 +1568,17 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
-      <c r="P6" s="2" t="s">
-        <v>20</v>
+      <c r="P6" t="s">
+        <v>26</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="R6" s="2"/>
     </row>
     <row r="7" spans="1:18">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>8</v>
@@ -1581,7 +1587,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>24</v>
@@ -1594,11 +1600,11 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-      <c r="P7" s="2" t="s">
-        <v>25</v>
+      <c r="P7" t="s">
+        <v>29</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="R7" s="2"/>
     </row>
@@ -1626,8 +1632,12 @@
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
+      <c r="P8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="R8" s="2"/>
     </row>
     <row r="9" spans="1:18">
@@ -1654,8 +1664,12 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
+      <c r="P9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="R9" s="2"/>
     </row>
     <row r="10" spans="1:18">
@@ -1674,8 +1688,6 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
     </row>
     <row r="11" spans="1:18">
@@ -1720,21 +1732,21 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -1831,13 +1843,13 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -1858,7 +1870,7 @@
     </row>
     <row r="17" spans="1:18">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
@@ -1878,7 +1890,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>8</v>
@@ -1903,7 +1915,7 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>24</v>
@@ -1912,7 +1924,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>8</v>
@@ -1928,7 +1940,7 @@
     </row>
     <row r="19" spans="1:18">
       <c r="A19" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>24</v>
@@ -1937,7 +1949,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>14</v>

</xml_diff>